<commit_message>
feat(product-groups): re-walk the list page to depth and give each sub-task its own case sequence (NM-2258, NM-2259)
NM-2258 — Search For Product Groups: deep re-walk of the list page (2026-09-09 inventory, evidence under .playwright-cli/pgr-2026-09-09/); 32 cases added for 39 in total; three defects filed (BUG-ISR-PGR-001/002/003); TC-ISR-PGR-016 fails on purpose as the evidence for the search-debounce defect.

NM-2259 — Create new Product Groups: corrections from the family run (description uniqueness is NM-1851's rule; rejection toasts expire after about 10 s); cases unchanged in substance.

Phase 9 (owner-directed): one contiguous case sequence per sub-task — TC-ISR-PGR-001…039 in spec order, TC-ISR-APG-001…023 under the Add page's own code; registry, manifest tc_ids, workbooks, inventories, bugs and plans carried along. No push.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/encore/testcases/create-new-product-groups/item-search-create-new-product-groups.xlsx
+++ b/clients/encore/testcases/create-new-product-groups/item-search-create-new-product-groups.xlsx
@@ -52,7 +52,7 @@
     <t>Notes / Reason</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-006</t>
+    <t>TC-ISR-APG-001</t>
   </si>
   <si>
     <t>The Add page opens with a held-back Save</t>
@@ -111,7 +111,7 @@
     <t>Save stays disabled — the other required fields are still empty</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-007</t>
+    <t>TC-ISR-APG-002</t>
   </si>
   <si>
     <t>The sub-class picker shows its two panels</t>
@@ -132,7 +132,7 @@
     <t>It is marked required and shows the instruction "Drag or double‑click items from the left to add sub‑classes"</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-008</t>
+    <t>TC-ISR-APG-003</t>
   </si>
   <si>
     <t>Cancel leaves the Add page without saving</t>
@@ -153,7 +153,7 @@
     <t>The form is empty again; nothing was kept</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-011</t>
+    <t>TC-ISR-APG-004</t>
   </si>
   <si>
     <t>A completed Add page saves a new product group and it is found again</t>
@@ -192,7 +192,7 @@
     <t>Exactly one row returns — the group just created, showing its Description and Service Type</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-012</t>
+    <t>TC-ISR-APG-005</t>
   </si>
   <si>
     <t>Name accepts exactly 50 characters and drops the rest silently</t>
@@ -231,7 +231,7 @@
     <t>The list page returns; nothing was saved</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-013</t>
+    <t>TC-ISR-APG-006</t>
   </si>
   <si>
     <t>Description accepts exactly 100 characters and drops the rest silently</t>
@@ -255,7 +255,7 @@
     <t>4. Click Cancel</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-014</t>
+    <t>TC-ISR-APG-007</t>
   </si>
   <si>
     <t>Clearing a filled Name by either method holds Save back and marks the box invalid</t>
@@ -297,7 +297,7 @@
     <t>6. Click Cancel</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-015</t>
+    <t>TC-ISR-APG-008</t>
   </si>
   <si>
     <t>A whitespace-only Name counts as empty; a padded Name is accepted</t>
@@ -321,7 +321,7 @@
     <t>3. Click Cancel</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-016</t>
+    <t>TC-ISR-APG-009</t>
   </si>
   <si>
     <t>Every required field gates Save, and Active does not</t>
@@ -363,7 +363,7 @@
     <t>8. Click Cancel</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-017</t>
+    <t>TC-ISR-APG-010</t>
   </si>
   <si>
     <t>The Service Type list offers its 90 options with no search box, and first, middle and last all select</t>
@@ -399,7 +399,7 @@
     <t>The selector shows "Lighting"</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-018</t>
+    <t>TC-ISR-APG-011</t>
   </si>
   <si>
     <t>A name already used by another group is rejected, with or without a trailing space</t>
@@ -426,7 +426,7 @@
     <t>The list page returns; nothing was created</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-019</t>
+    <t>TC-ISR-APG-012</t>
   </si>
   <si>
     <t>A description already used by another group is rejected even with a new name</t>
@@ -438,7 +438,7 @@
     <t>An error toast reads `Product group name '&lt;the new name&gt;' or group description 'walk probe A' already exists.`; the page stays on the Add form; Save is still enabled</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-020</t>
+    <t>TC-ISR-APG-013</t>
   </si>
   <si>
     <t>The picker search filters the catalog by substring regardless of case and empties on no match</t>
@@ -484,7 +484,7 @@
     <t>The list page returns</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-021</t>
+    <t>TC-ISR-APG-014</t>
   </si>
   <si>
     <t>The Labor filter narrows the catalog and unchecking restores it</t>
@@ -508,7 +508,7 @@
     <t>The count and first row from step 1 return</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-022</t>
+    <t>TC-ISR-APG-015</t>
   </si>
   <si>
     <t>Sort order flips the catalog between ascending and descending</t>
@@ -532,7 +532,7 @@
     <t>Step 1's first and last rows return</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-023</t>
+    <t>TC-ISR-APG-016</t>
   </si>
   <si>
     <t>Reset clears the picker's search, filter and sort but keeps an added sub-class</t>
@@ -562,7 +562,7 @@
     <t>Search is empty, Labor is unchecked, the order shows Ascending, the full catalog is back — and the sub-class added in step 1 is still in the Sub Classes area</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-024</t>
+    <t>TC-ISR-APG-017</t>
   </si>
   <si>
     <t>Double-click adds an item once and the x control removes it</t>
@@ -586,7 +586,7 @@
     <t>The Sub Classes area is empty and the instruction text is back; the catalog is unchanged</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-025</t>
+    <t>TC-ISR-APG-018</t>
   </si>
   <si>
     <t>Dragging an item onto the Sub Classes area adds it</t>
@@ -604,7 +604,7 @@
     <t>2. Click Cancel</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-026</t>
+    <t>TC-ISR-APG-019</t>
   </si>
   <si>
     <t>The divider button collapses and expands the sub-class panel</t>
@@ -635,7 +635,7 @@
     <t>The button reads "Collapse search panel" again and the Name box has step 1's left edge and width</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-027</t>
+    <t>TC-ISR-APG-020</t>
   </si>
   <si>
     <t>A group saved with Active cleared is created inactive and found with the list's Active filter cleared</t>
@@ -662,7 +662,7 @@
     <t>5. Clear the Active filter and search again</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-028</t>
+    <t>TC-ISR-APG-021</t>
   </si>
   <si>
     <t>Special characters in the name are stored verbatim and the last Service Type saves</t>
@@ -686,7 +686,7 @@
     <t>4. Search the list for the new group</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-029</t>
+    <t>TC-ISR-APG-022</t>
   </si>
   <si>
     <t>Browser Back leaves the Add page without saving or warning</t>
@@ -713,7 +713,7 @@
     <t>The form is empty; nothing was kept</t>
   </si>
   <si>
-    <t>TC-ISR-PGR-030</t>
+    <t>TC-ISR-APG-023</t>
   </si>
   <si>
     <t>The breadcrumb leaves the Add page without saving or warning</t>
@@ -743,7 +743,7 @@
     <t>Pass:23 Fail:0 Skipped:0 Blocked:0</t>
   </si>
   <si>
-    <t>Last Updated: 2026-09-09</t>
+    <t>Last Updated: 2026-09-10</t>
   </si>
 </sst>
 </file>

</xml_diff>